<commit_message>
Add i18n to installer: 49 installer keys, auto-detect system language
Extends the same LanguageTranslator mechanism from the editor to the
installer GUI. A module-level _init_translator() resolves languages.xlsx
(dev path or PyInstaller _MEIPASS), detects the system input language via
get_current_input_language(), and returns a tr() callable that falls back
to the key if the xlsx is unavailable.

All visible strings in PMS_Installer are now translated: window title,
status labels, checkboxes, buttons, and all messagebox titles/bodies.
languages.xlsx gains 49 installer.* keys (English / 繁體中文 / 簡体中文).

build_installer.py bundles languages.xlsx via --add-data and adds
hidden imports for py_libraries, pandas, openpyxl so they survive
PyInstaller tree-shaking.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pms/editor/languages.xlsx
+++ b/pms/editor/languages.xlsx
@@ -2,27 +2,33 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="2160" yWindow="0" windowWidth="16220" windowHeight="13952" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="translations" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
-      <name val="Calibri"/>
+      <name val="新細明體"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="新細明體"/>
+      <charset val="136"/>
+      <family val="3"/>
+      <sz val="9"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -50,7 +56,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="一般" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -413,8 +419,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D113"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:D162"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.95"/>
+  <cols>
+    <col width="27.5" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="25.125" customWidth="1" min="3" max="3"/>
+    <col width="32.875" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1001,12 +1013,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>個事件</t>
+          <t>事件數量</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>个事件</t>
+          <t>事件数量</t>
         </is>
       </c>
     </row>
@@ -1023,12 +1035,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>個片段</t>
+          <t>片段數量</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>个片段</t>
+          <t>片段数量</t>
         </is>
       </c>
     </row>
@@ -1045,12 +1057,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>個概念</t>
+          <t>概念數量</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>个概念</t>
+          <t>概念数量</t>
         </is>
       </c>
     </row>
@@ -1067,12 +1079,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>個結果</t>
+          <t>結果數量</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>个结果</t>
+          <t>结果数量</t>
         </is>
       </c>
     </row>
@@ -2899,6 +2911,1108 @@
       <c r="D113" t="inlineStr">
         <is>
           <t>加载</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>installer.window_title</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Installer</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>安裝程式</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>安装程序</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>installer.installed_at</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>is installed at</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>已安裝於</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>已安装于</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>installer.not_installed</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>is not installed</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>尚未安裝</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>尚未安装</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>installer.options</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Options</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>選項</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>选项</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>installer.create_shortcut</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Create desktop shortcut for PMS Editor</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>建立 PMS 編輯器桌面捷徑</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>创建 PMS 编辑器桌面快捷方式</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>installer.setup_ollama</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Set up Ollama and pull models</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>設定 Ollama 並拉取模型</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>设置 Ollama 并拉取模型</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>installer.launch_after</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Launch editor after install</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>安裝後啟動編輯器</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>安装后启动编辑器</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>installer.btn_install</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Install</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>安裝</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>安装</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>installer.btn_reinstall</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Reinstall</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>重新安裝</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>重新安装</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>installer.btn_uninstall</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Uninstall</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>解除安裝</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>卸载</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>installer.btn_exit</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Exit</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>結束</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>退出</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>installer.stopping_svc</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Stopping previous PMS services…</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>停止現有 PMS 服務…</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>停止现有 PMS 服务…</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>installer.preparing_dir</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Preparing install directory…</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>準備安裝目錄…</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>准备安装目录…</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>installer.copying_files</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Copying files…</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>複製檔案…</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>复制文件…</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>installer.adding_path</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Adding PMS to PATH…</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>將 PMS 加入 PATH…</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>将 PMS 加入 PATH…</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>installer.installing_svc</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Installing Windows service…</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>安裝 Windows 服務…</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>安装 Windows 服务…</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>installer.downloading_nssm</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Downloading NSSM…</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>下載 NSSM…</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>下载 NSSM…</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>installer.nssm_failed</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>NSSM download failed</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>NSSM 下載失敗</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>NSSM 下载失败</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>installer.creating_shortcut</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Creating desktop shortcut…</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>建立桌面捷徑…</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>创建桌面快捷方式…</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>installer.complete</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Installation complete.</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>安裝完成。</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>安装完成。</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>installer.failed</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Installation failed.</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>安裝失敗。</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>安装失败。</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>installer.skipping_ollama</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Skipping model pull — Ollama not available.</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>跳過模型拉取 — Ollama 不可用。</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>跳过模型拉取 — Ollama 不可用。</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>installer.already_present</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>already present — skipping.</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>已存在，略過。</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>已存在，跳过。</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>installer.pulling_model</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Pulling</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>拉取</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>拉取</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>installer.downloading_ollama</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Downloading Ollama installer…</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>下載 Ollama 安裝程式…</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>下载 Ollama 安装程序…</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>installer.installing_ollama</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Installing Ollama…</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>安裝 Ollama…</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>安装 Ollama…</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>installer.ollama_failed</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Ollama install failed</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Ollama 安裝失敗</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Ollama 安装失败</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>installer.svc_running</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>The PMS server is running on http://127.0.0.1:8765</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>PMS 伺服器正在 http://127.0.0.1:8765 執行</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>PMS 服务器正在 http://127.0.0.1:8765 运行</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>installer.svc_not_installed</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Start pms_server.exe manually (NSSM service not installed).</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>請手動啟動 pms_server.exe（NSSM 服務未安裝）。</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>请手动启动 pms_server.exe（NSSM 服务未安装）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>installer.path_notice</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>PMS has been added to your PATH. Open a new terminal to run 'pms_manager status' from anywhere.</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>PMS 已加入 PATH。開啟新終端機即可在任何位置執行 pms_manager status。</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>PMS 已加入 PATH。打开新终端即可在任何位置运行 pms_manager status。</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>installer.uninstalling_svc</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Stopping and removing service…</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>停止並移除服務…</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>停止并移除服务…</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>installer.removing_path</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Removing PMS from PATH…</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>從 PATH 移除 PMS…</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>从 PATH 移除 PMS…</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>installer.removing_shortcut</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Removing desktop shortcut…</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>移除桌面捷徑…</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>移除桌面快捷方式…</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>installer.removing_files</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Removing files…</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>移除檔案…</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>移除文件…</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>installer.done</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Done.</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>完成。</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>完成。</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>installer.msg_admin_title</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Administrator Required</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>需要管理員權限</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>需要管理员权限</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>installer.msg_admin_body</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Please run the installer as Administrator
+(required for Windows service installation).</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>請以管理員身份執行安裝程式
+（安裝 Windows 服務所必需）。</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>请以管理员身份运行安装程序
+（安装 Windows 服务所必需）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>installer.msg_svc_title</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Service Not Installed</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>服務未安裝</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>服务未安装</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>installer.msg_svc_body</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>NSSM could not be found or downloaded — the Windows service was not installed.
+Download NSSM from https://nssm.cc/download and add it to PATH,
+then re-run the installer.</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>找不到或無法下載 NSSM — Windows 服務未安裝。
+請從 https://nssm.cc/download 下載 NSSM 並加入 PATH，
+然後重新執行安裝程式。</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>找不到或无法下载 NSSM — Windows 服务未安装。
+请从 https://nssm.cc/download 下载 NSSM 并加入 PATH，
+然后重新运行安装程序。</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>installer.msg_complete_title</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Installation Complete</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>安裝完成</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>安装完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>installer.msg_uninstall_confirm_title</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Confirm Uninstall</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>確認解除安裝</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>确认卸载</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>installer.msg_uninstall_confirm_body</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Uninstall {app}?
+config.yaml will be preserved.</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>解除安裝 {app}？
+config.yaml 將會保留。</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>卸载 {app}？
+config.yaml 将被保留。</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>installer.msg_uninstalled_title</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Uninstalled</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>已解除安裝</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>已卸载</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>installer.msg_uninstalled_body</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>has been uninstalled.
+config.yaml has been preserved at:</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>已解除安裝。
+config.yaml 已保留於：</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>已卸载。
+config.yaml 已保留于：</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>installer.msg_uninstall_error</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Uninstall Error</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>解除安裝錯誤</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>卸载错误</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>installer.msg_install_error</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Installation Error</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>安裝錯誤</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>安装错误</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>installer.msg_ollama_title</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Ollama Not Found</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>找不到 Ollama</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>找不到 Ollama</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>installer.msg_ollama_body</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Ollama is not installed.
+Download and install it now? (~100 MB)
+Ollama powers AI consolidation and vector search.
+PMS works without it — retrieval falls back to keyword search only.</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>未安裝 Ollama。
+立即下載並安裝？（約 100 MB）
+Ollama 提供 AI 整合與向量搜尋功能。
+沒有也可以使用 PMS — 搜尋將回退至關鍵字模式。</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>未安装 Ollama。
+立即下载并安装？（约 100 MB）
+Ollama 提供 AI 整合与向量搜索功能。
+没有也可以使用 PMS — 搜索将回退至关键词模式。</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>installer.msg_ollama_fail_title</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Ollama Install Failed</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Ollama 安裝失敗</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Ollama 安装失败</t>
         </is>
       </c>
     </row>

</xml_diff>